<commit_message>
added pairwise with vpol dependant of R.
</commit_message>
<xml_diff>
--- a/scripts_python/references/data_pair.xlsx
+++ b/scripts_python/references/data_pair.xlsx
@@ -165,15 +165,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
 </styleSheet>
 </file>
 
@@ -421,772 +412,772 @@
       <c r="A4" s="2" t="n">
         <v>0.377268211971313</v>
       </c>
-      <c r="B4" s="0" t="n">
-        <v>-43.1575218741381</v>
-      </c>
-      <c r="C4" s="0" t="n">
+      <c r="B4" s="2" t="n">
+        <v>-42.7056057085545</v>
+      </c>
+      <c r="C4" s="2" t="n">
         <v>0.402246234516001</v>
       </c>
-      <c r="D4" s="0" t="n">
-        <v>143.462689614481</v>
+      <c r="D4" s="2" t="n">
+        <v>143.332940604161</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0.402246234516001</v>
       </c>
-      <c r="F4" s="0" t="n">
-        <v>208.790323617338</v>
-      </c>
-      <c r="G4" s="0" t="n">
+      <c r="F4" s="2" t="n">
+        <v>199.589579900542</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>0.377268211971313</v>
       </c>
-      <c r="H4" s="0" t="n">
-        <v>14.0070166354753</v>
-      </c>
-      <c r="I4" s="0" t="n">
+      <c r="H4" s="2" t="n">
+        <v>13.8503417826426</v>
+      </c>
+      <c r="I4" s="2" t="n">
         <v>0.501745677347789</v>
       </c>
-      <c r="J4" s="0" t="n">
-        <v>29.9653928920374</v>
-      </c>
-      <c r="K4" s="0" t="n">
+      <c r="J4" s="2" t="n">
+        <v>29.8891981345111</v>
+      </c>
+      <c r="K4" s="2" t="n">
         <v>0.377268211971313</v>
       </c>
-      <c r="L4" s="0" t="n">
-        <v>-17.0566398801337</v>
-      </c>
-      <c r="M4" s="0" t="n">
+      <c r="L4" s="2" t="n">
+        <v>-16.7425686143361</v>
+      </c>
+      <c r="M4" s="2" t="n">
         <v>0.402246234516001</v>
       </c>
-      <c r="N4" s="0" t="n">
-        <v>143.460259614715</v>
-      </c>
-      <c r="O4" s="0" t="n">
+      <c r="N4" s="2" t="n">
+        <v>143.330307961806</v>
+      </c>
+      <c r="O4" s="2" t="n">
         <v>0.402246234516001</v>
       </c>
-      <c r="P4" s="0" t="n">
-        <v>41.6817150296412</v>
-      </c>
-      <c r="Q4" s="0" t="n">
+      <c r="P4" s="2" t="n">
+        <v>41.4883113107771</v>
+      </c>
+      <c r="Q4" s="2" t="n">
         <v>0.377268211971313</v>
       </c>
-      <c r="R4" s="0" t="n">
-        <v>4.12168580941952</v>
-      </c>
-      <c r="S4" s="0" t="n">
+      <c r="R4" s="2" t="n">
+        <v>4.17028023085523</v>
+      </c>
+      <c r="S4" s="2" t="n">
         <v>0.377268211971313</v>
       </c>
-      <c r="T4" s="0" t="n">
-        <v>-13.3420359177118</v>
-      </c>
-      <c r="U4" s="0" t="n">
+      <c r="T4" s="2" t="n">
+        <v>-13.2812255836668</v>
+      </c>
+      <c r="U4" s="2" t="n">
         <v>0.402246234516001</v>
       </c>
-      <c r="V4" s="0" t="n">
-        <v>44.2372257094628</v>
-      </c>
-      <c r="W4" s="0" t="n">
+      <c r="V4" s="2" t="n">
+        <v>44.1057834829935</v>
+      </c>
+      <c r="W4" s="2" t="n">
         <v>0.402246234516001</v>
       </c>
-      <c r="X4" s="0" t="n">
-        <v>-17.4030978629346</v>
-      </c>
-      <c r="Y4" s="0" t="n">
+      <c r="X4" s="2" t="n">
+        <v>-17.1585190912514</v>
+      </c>
+      <c r="Y4" s="2" t="n">
         <v>0.402246234516001</v>
       </c>
-      <c r="Z4" s="0" t="n">
-        <v>21.111717064205</v>
+      <c r="Z4" s="2" t="n">
+        <v>20.7605211695015</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="n">
+        <v>0.45058944405295</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>-46.797205844243</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>0.501745677347789</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>99.2570696380353</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0.501745677347789</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>184.509360861422</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0.45058944405295</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>-15.2666963315436</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0.599313443125452</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>-2.54443763053527</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>0.45058944405295</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>12.0949143326211</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>0.501745677347789</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>99.2529899240402</v>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>0.501745677347789</v>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>55.2636775928942</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>0.45058944405295</v>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>4.91920360623092</v>
+      </c>
+      <c r="S5" s="2" t="n">
         <v>0.402246234516001</v>
       </c>
-      <c r="B5" s="0" t="n">
-        <v>-46.8739732838978</v>
-      </c>
-      <c r="C5" s="0" t="n">
-        <v>0.45058944405295</v>
-      </c>
-      <c r="D5" s="0" t="n">
-        <v>124.069521177372</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>0.45058944405295</v>
-      </c>
-      <c r="F5" s="0" t="n">
-        <v>201.686793427728</v>
-      </c>
-      <c r="G5" s="0" t="n">
-        <v>0.402246234516001</v>
-      </c>
-      <c r="H5" s="0" t="n">
-        <v>2.63227314619222</v>
-      </c>
-      <c r="I5" s="0" t="n">
-        <v>0.551214899264904</v>
-      </c>
-      <c r="J5" s="0" t="n">
-        <v>13.8356891621664</v>
-      </c>
-      <c r="K5" s="0" t="n">
-        <v>0.402246234516001</v>
-      </c>
-      <c r="L5" s="0" t="n">
-        <v>-10.7727249664519</v>
-      </c>
-      <c r="M5" s="0" t="n">
-        <v>0.45058944405295</v>
-      </c>
-      <c r="N5" s="0" t="n">
-        <v>124.065053820864</v>
-      </c>
-      <c r="O5" s="0" t="n">
-        <v>0.45058944405295</v>
-      </c>
-      <c r="P5" s="0" t="n">
-        <v>46.0597521731339</v>
-      </c>
-      <c r="Q5" s="0" t="n">
-        <v>0.402246234516001</v>
-      </c>
-      <c r="R5" s="0" t="n">
-        <v>4.55685802541893</v>
-      </c>
-      <c r="S5" s="0" t="n">
-        <v>0.402246234516001</v>
-      </c>
-      <c r="T5" s="0" t="n">
-        <v>-21.2018708449674</v>
-      </c>
-      <c r="U5" s="0" t="n">
-        <v>0.45058944405295</v>
-      </c>
-      <c r="V5" s="0" t="n">
-        <v>55.9689917803121</v>
-      </c>
-      <c r="W5" s="0" t="n">
-        <v>0.45058944405295</v>
-      </c>
-      <c r="X5" s="0" t="n">
-        <v>-11.0217591713346</v>
-      </c>
-      <c r="Y5" s="0" t="n">
-        <v>0.45058944405295</v>
-      </c>
-      <c r="Z5" s="0" t="n">
-        <v>14.0380305994736</v>
+      <c r="T5" s="2" t="n">
+        <v>-21.0706217446609</v>
+      </c>
+      <c r="U5" s="2" t="n">
+        <v>0.501745677347789</v>
+      </c>
+      <c r="V5" s="2" t="n">
+        <v>86.2307108061334</v>
+      </c>
+      <c r="W5" s="2" t="n">
+        <v>0.501745677347789</v>
+      </c>
+      <c r="X5" s="2" t="n">
+        <v>1.45255144215534</v>
+      </c>
+      <c r="Y5" s="2" t="n">
+        <v>0.501745677347789</v>
+      </c>
+      <c r="Z5" s="2" t="n">
+        <v>4.28943953319259</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="n">
+        <v>0.551214899264904</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>-19.628396931761</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0.599313443125452</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>50.3437223376037</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0.599313443125452</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>108.914507978603</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0.551214899264904</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>-36.5716829603238</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0.650493343520364</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>-12.7691400693566</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>0.551214899264904</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>74.6244139616082</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>0.599313443125452</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>50.3432488912148</v>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>0.599313443125452</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>67.5994172460176</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>0.551214899264904</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>-9.79249149755205</v>
+      </c>
+      <c r="S6" s="2" t="n">
         <v>0.45058944405295</v>
       </c>
-      <c r="B6" s="0" t="n">
-        <v>-47.348019890578</v>
-      </c>
-      <c r="C6" s="0" t="n">
-        <v>0.501745677347789</v>
-      </c>
-      <c r="D6" s="0" t="n">
-        <v>99.4273374570692</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>0.501745677347789</v>
-      </c>
-      <c r="F6" s="0" t="n">
-        <v>184.743501344904</v>
-      </c>
-      <c r="G6" s="0" t="n">
-        <v>0.45058944405295</v>
-      </c>
-      <c r="H6" s="0" t="n">
-        <v>-15.3761606649351</v>
-      </c>
-      <c r="I6" s="0" t="n">
+      <c r="T6" s="2" t="n">
+        <v>-24.3074411517975</v>
+      </c>
+      <c r="U6" s="2" t="n">
         <v>0.599313443125452</v>
       </c>
-      <c r="J6" s="0" t="n">
-        <v>-2.53300904262687</v>
-      </c>
-      <c r="K6" s="0" t="n">
-        <v>0.45058944405295</v>
-      </c>
-      <c r="L6" s="0" t="n">
-        <v>11.7146976026923</v>
-      </c>
-      <c r="M6" s="0" t="n">
-        <v>0.501745677347789</v>
-      </c>
-      <c r="N6" s="0" t="n">
-        <v>99.4231120009112</v>
-      </c>
-      <c r="O6" s="0" t="n">
-        <v>0.501745677347789</v>
-      </c>
-      <c r="P6" s="0" t="n">
-        <v>55.5196370927983</v>
-      </c>
-      <c r="Q6" s="0" t="n">
-        <v>0.45058944405295</v>
-      </c>
-      <c r="R6" s="0" t="n">
-        <v>4.90005930171654</v>
-      </c>
-      <c r="S6" s="0" t="n">
-        <v>0.45058944405295</v>
-      </c>
-      <c r="T6" s="0" t="n">
-        <v>-24.5566758350907</v>
-      </c>
-      <c r="U6" s="0" t="n">
-        <v>0.501745677347789</v>
-      </c>
-      <c r="V6" s="0" t="n">
-        <v>86.2999464687387</v>
-      </c>
-      <c r="W6" s="0" t="n">
-        <v>0.501745677347789</v>
-      </c>
-      <c r="X6" s="0" t="n">
-        <v>1.23799098248358</v>
-      </c>
-      <c r="Y6" s="0" t="n">
-        <v>0.501745677347789</v>
-      </c>
-      <c r="Z6" s="0" t="n">
-        <v>14.7555768893566</v>
+      <c r="V6" s="2" t="n">
+        <v>183.135689236163</v>
+      </c>
+      <c r="W6" s="2" t="n">
+        <v>0.599313443125452</v>
+      </c>
+      <c r="X6" s="2" t="n">
+        <v>30.0541501512625</v>
+      </c>
+      <c r="Y6" s="2" t="n">
+        <v>0.599313443125452</v>
+      </c>
+      <c r="Z6" s="2" t="n">
+        <v>11.5162547431741</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="n">
+        <v>0.650493343520364</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>54.6753599677365</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0.700545785025913</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>18.2800038506729</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>0.700545785025913</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>9.43971861035774</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.650493343520364</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>-12.2767997596666</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0.700545785025913</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>-15.2711131605406</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>0.650493343520364</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>105.470054729041</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>0.700545785025913</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>18.2807198851496</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>0.700545785025913</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>65.7096505528434</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>0.650493343520364</v>
+      </c>
+      <c r="R7" s="2" t="n">
+        <v>-13.434164226217</v>
+      </c>
+      <c r="S7" s="2" t="n">
         <v>0.501745677347789</v>
       </c>
-      <c r="B7" s="0" t="n">
-        <v>-38.5813555465901</v>
-      </c>
-      <c r="C7" s="0" t="n">
-        <v>0.551214899264904</v>
-      </c>
-      <c r="D7" s="0" t="n">
-        <v>73.7821637175288</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>0.551214899264904</v>
-      </c>
-      <c r="F7" s="0" t="n">
-        <v>152.684276475048</v>
-      </c>
-      <c r="G7" s="0" t="n">
-        <v>0.501745677347789</v>
-      </c>
-      <c r="H7" s="0" t="n">
-        <v>-29.641012816477</v>
-      </c>
-      <c r="I7" s="0" t="n">
-        <v>0.625057060568896</v>
-      </c>
-      <c r="J7" s="0" t="n">
-        <v>-9.14763977143551</v>
-      </c>
-      <c r="K7" s="0" t="n">
-        <v>0.501745677347789</v>
-      </c>
-      <c r="L7" s="0" t="n">
-        <v>43.219283182032</v>
-      </c>
-      <c r="M7" s="0" t="n">
-        <v>0.551214899264904</v>
-      </c>
-      <c r="N7" s="0" t="n">
-        <v>73.7786689045187</v>
-      </c>
-      <c r="O7" s="0" t="n">
-        <v>0.551214899264904</v>
-      </c>
-      <c r="P7" s="0" t="n">
-        <v>63.5442937980272</v>
-      </c>
-      <c r="Q7" s="0" t="n">
-        <v>0.501745677347789</v>
-      </c>
-      <c r="R7" s="0" t="n">
-        <v>-1.37998743131934</v>
-      </c>
-      <c r="S7" s="0" t="n">
-        <v>0.501745677347789</v>
-      </c>
-      <c r="T7" s="0" t="n">
-        <v>-11.1503540175822</v>
-      </c>
-      <c r="U7" s="0" t="n">
-        <v>0.551214899264904</v>
-      </c>
-      <c r="V7" s="0" t="n">
-        <v>129.263706069386</v>
-      </c>
-      <c r="W7" s="0" t="n">
-        <v>0.551214899264904</v>
-      </c>
-      <c r="X7" s="0" t="n">
-        <v>13.5158618496915</v>
-      </c>
-      <c r="Y7" s="0" t="n">
-        <v>0.551214899264904</v>
-      </c>
-      <c r="Z7" s="0" t="n">
-        <v>22.3980795913511</v>
+      <c r="T7" s="2" t="n">
+        <v>-10.8127338642822</v>
+      </c>
+      <c r="U7" s="2" t="n">
+        <v>0.700545785025913</v>
+      </c>
+      <c r="V7" s="2" t="n">
+        <v>270.757938095879</v>
+      </c>
+      <c r="W7" s="2" t="n">
+        <v>0.700545785025913</v>
+      </c>
+      <c r="X7" s="2" t="n">
+        <v>119.064821308219</v>
+      </c>
+      <c r="Y7" s="2" t="n">
+        <v>0.700545785025913</v>
+      </c>
+      <c r="Z7" s="2" t="n">
+        <v>70.7804658279231</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="n">
+        <v>0.402246234516001</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>-46.3802292370815</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>0.761787315617629</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>18.1391269667533</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>0.801917215853616</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>-35.0016883411335</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0.402246234516001</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>2.54605846866311</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0.801917215853616</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>23.9178656431647</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>0.402246234516001</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>-10.4354255326404</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>0.801917215853616</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>32.0056417872096</v>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>0.801917215853616</v>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>51.583005157292</v>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>0.402246234516001</v>
+      </c>
+      <c r="R8" s="2" t="n">
+        <v>4.60436515574824</v>
+      </c>
+      <c r="S8" s="2" t="n">
         <v>0.551214899264904</v>
       </c>
-      <c r="B8" s="0" t="n">
-        <v>-20.1448774299834</v>
-      </c>
-      <c r="C8" s="0" t="n">
-        <v>0.599313443125452</v>
-      </c>
-      <c r="D8" s="0" t="n">
-        <v>50.5732455542331</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>0.599313443125452</v>
-      </c>
-      <c r="F8" s="0" t="n">
-        <v>109.22265544432</v>
-      </c>
-      <c r="G8" s="0" t="n">
-        <v>0.551214899264904</v>
-      </c>
-      <c r="H8" s="0" t="n">
-        <v>-36.9476705450046</v>
-      </c>
-      <c r="I8" s="0" t="n">
-        <v>0.650493343520364</v>
-      </c>
-      <c r="J8" s="0" t="n">
-        <v>-12.8447286919134</v>
-      </c>
-      <c r="K8" s="0" t="n">
-        <v>0.551214899264904</v>
-      </c>
-      <c r="L8" s="0" t="n">
-        <v>74.2835197491118</v>
-      </c>
-      <c r="M8" s="0" t="n">
-        <v>0.599313443125452</v>
-      </c>
-      <c r="N8" s="0" t="n">
-        <v>50.5724364092023</v>
-      </c>
-      <c r="O8" s="0" t="n">
-        <v>0.599313443125452</v>
-      </c>
-      <c r="P8" s="0" t="n">
-        <v>67.9449730022091</v>
-      </c>
-      <c r="Q8" s="0" t="n">
-        <v>0.551214899264904</v>
-      </c>
-      <c r="R8" s="0" t="n">
-        <v>-9.77770908098958</v>
-      </c>
-      <c r="S8" s="0" t="n">
-        <v>0.551214899264904</v>
-      </c>
-      <c r="T8" s="0" t="n">
-        <v>21.0985912796597</v>
-      </c>
-      <c r="U8" s="0" t="n">
-        <v>0.599313443125452</v>
-      </c>
-      <c r="V8" s="0" t="n">
-        <v>183.367394932493</v>
-      </c>
-      <c r="W8" s="0" t="n">
-        <v>0.599313443125452</v>
-      </c>
-      <c r="X8" s="0" t="n">
-        <v>30.0580845025508</v>
-      </c>
-      <c r="Y8" s="0" t="n">
-        <v>0.599313443125452</v>
-      </c>
-      <c r="Z8" s="0" t="n">
-        <v>37.9083587049103</v>
+      <c r="T8" s="2" t="n">
+        <v>21.443536560276</v>
+      </c>
+      <c r="U8" s="2" t="n">
+        <v>0.45058944405295</v>
+      </c>
+      <c r="V8" s="2" t="n">
+        <v>55.9010314965605</v>
+      </c>
+      <c r="W8" s="2" t="n">
+        <v>0.45058944405295</v>
+      </c>
+      <c r="X8" s="2" t="n">
+        <v>-10.7463340909484</v>
+      </c>
+      <c r="Y8" s="2" t="n">
+        <v>0.45058944405295</v>
+      </c>
+      <c r="Z8" s="2" t="n">
+        <v>10.3741949377648</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="n">
+        <v>0.501745677347789</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>-38.0162512055716</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>0.849436782010227</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>34.3761508168014</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>0.900227517476009</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>6.58876088932669</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.501745677347789</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>-29.3609074030252</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0.551214899264904</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>13.7470290968536</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>0.501745677347789</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>43.6351725449249</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>0.900227517476009</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>29.0126632167253</v>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>0.900227517476009</v>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>18.4039618058375</v>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>0.501745677347789</v>
+      </c>
+      <c r="R9" s="2" t="n">
+        <v>-1.42050937432677</v>
+      </c>
+      <c r="S9" s="2" t="n">
         <v>0.599313443125452</v>
       </c>
-      <c r="B9" s="0" t="n">
-        <v>9.34472612440317</v>
-      </c>
-      <c r="C9" s="0" t="n">
-        <v>0.650493343520364</v>
-      </c>
-      <c r="D9" s="0" t="n">
-        <v>30.5732815751131</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>0.650493343520364</v>
-      </c>
-      <c r="F9" s="0" t="n">
-        <v>56.4016104619132</v>
-      </c>
-      <c r="G9" s="0" t="n">
-        <v>0.599313443125452</v>
-      </c>
-      <c r="H9" s="0" t="n">
-        <v>-36.9272034808634</v>
-      </c>
-      <c r="I9" s="0" t="n">
-        <v>0.675648581248717</v>
-      </c>
-      <c r="J9" s="0" t="n">
-        <v>-16.1546776987763</v>
-      </c>
-      <c r="K9" s="0" t="n">
-        <v>0.599313443125452</v>
-      </c>
-      <c r="L9" s="0" t="n">
-        <v>97.6294742076894</v>
-      </c>
-      <c r="M9" s="0" t="n">
-        <v>0.650493343520364</v>
-      </c>
-      <c r="N9" s="0" t="n">
-        <v>30.5732841689381</v>
-      </c>
-      <c r="O9" s="0" t="n">
-        <v>0.650493343520364</v>
-      </c>
-      <c r="P9" s="0" t="n">
-        <v>68.0408498783784</v>
-      </c>
-      <c r="Q9" s="0" t="n">
-        <v>0.599313443125452</v>
-      </c>
-      <c r="R9" s="0" t="n">
-        <v>-15.0269515473568</v>
-      </c>
-      <c r="S9" s="0" t="n">
-        <v>0.599313443125452</v>
-      </c>
-      <c r="T9" s="0" t="n">
-        <v>74.0512116398988</v>
-      </c>
-      <c r="U9" s="0" t="n">
-        <v>0.650493343520364</v>
-      </c>
-      <c r="V9" s="0" t="n">
-        <v>243.893904075153</v>
-      </c>
-      <c r="W9" s="0" t="n">
-        <v>0.650493343520364</v>
-      </c>
-      <c r="X9" s="0" t="n">
-        <v>62.9575691434977</v>
-      </c>
-      <c r="Y9" s="0" t="n">
-        <v>0.650493343520364</v>
-      </c>
-      <c r="Z9" s="0" t="n">
-        <v>63.5465237629709</v>
+      <c r="T9" s="2" t="n">
+        <v>74.2136712658181</v>
+      </c>
+      <c r="U9" s="2" t="n">
+        <v>0.551214899264904</v>
+      </c>
+      <c r="V9" s="2" t="n">
+        <v>129.136731509183</v>
+      </c>
+      <c r="W9" s="2" t="n">
+        <v>0.551214899264904</v>
+      </c>
+      <c r="X9" s="2" t="n">
+        <v>13.5864270476729</v>
+      </c>
+      <c r="Y9" s="2" t="n">
+        <v>0.551214899264904</v>
+      </c>
+      <c r="Z9" s="2" t="n">
+        <v>4.04074670263225</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="n">
+        <v>0.599313443125452</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>9.74493072222941</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>0.950390241271653</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>56.3545447747987</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>149.507913685346</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0.599313443125452</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>-36.5084067848157</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>0.625057060568896</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>-9.09918033975552</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>0.599313443125452</v>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>97.7073734351155</v>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>-0.0390590152805999</v>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>-0.0390590152805999</v>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>0.599313443125452</v>
+      </c>
+      <c r="R10" s="2" t="n">
+        <v>-15.0153999524053</v>
+      </c>
+      <c r="S10" s="2" t="n">
         <v>0.650493343520364</v>
       </c>
-      <c r="B10" s="0" t="n">
-        <v>54.4613501032256</v>
-      </c>
-      <c r="C10" s="0" t="n">
-        <v>0.700545785025913</v>
-      </c>
-      <c r="D10" s="0" t="n">
-        <v>18.5667820478967</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>0.700545785025913</v>
-      </c>
-      <c r="F10" s="0" t="n">
-        <v>9.55412804395641</v>
-      </c>
-      <c r="G10" s="0" t="n">
+      <c r="T10" s="2" t="n">
+        <v>156.814967381298</v>
+      </c>
+      <c r="U10" s="2" t="n">
         <v>0.650493343520364</v>
       </c>
-      <c r="H10" s="0" t="n">
-        <v>-12.585846329561</v>
-      </c>
-      <c r="I10" s="0" t="n">
-        <v>0.700545785025913</v>
-      </c>
-      <c r="J10" s="0" t="n">
-        <v>-15.3906819790813</v>
-      </c>
-      <c r="K10" s="0" t="n">
+      <c r="V10" s="2" t="n">
+        <v>243.239118561681</v>
+      </c>
+      <c r="W10" s="2" t="n">
         <v>0.650493343520364</v>
       </c>
-      <c r="L10" s="0" t="n">
-        <v>105.74377704474</v>
-      </c>
-      <c r="M10" s="0" t="n">
-        <v>0.700545785025913</v>
-      </c>
-      <c r="N10" s="0" t="n">
-        <v>18.5676187117574</v>
-      </c>
-      <c r="O10" s="0" t="n">
-        <v>0.700545785025913</v>
-      </c>
-      <c r="P10" s="0" t="n">
-        <v>65.9635691403024</v>
-      </c>
-      <c r="Q10" s="0" t="n">
+      <c r="X10" s="2" t="n">
+        <v>62.9064346870403</v>
+      </c>
+      <c r="Y10" s="2" t="n">
         <v>0.650493343520364</v>
       </c>
-      <c r="R10" s="0" t="n">
-        <v>-13.4340232774028</v>
-      </c>
-      <c r="S10" s="0" t="n">
-        <v>0.650493343520364</v>
-      </c>
-      <c r="T10" s="0" t="n">
-        <v>157.038204573064</v>
-      </c>
-      <c r="U10" s="0" t="n">
-        <v>0.700545785025913</v>
-      </c>
-      <c r="V10" s="0" t="n">
-        <v>271.69665731901</v>
-      </c>
-      <c r="W10" s="0" t="n">
-        <v>0.700545785025913</v>
-      </c>
-      <c r="X10" s="0" t="n">
-        <v>119.230330021196</v>
-      </c>
-      <c r="Y10" s="0" t="n">
-        <v>0.700545785025913</v>
-      </c>
-      <c r="Z10" s="0" t="n">
-        <v>97.2863536240173</v>
+      <c r="Z10" s="2" t="n">
+        <v>31.5133951049832</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="n">
         <v>0.700545785025913</v>
       </c>
-      <c r="B11" s="0" t="n">
-        <v>113.038826085836</v>
-      </c>
-      <c r="C11" s="0" t="n">
+      <c r="B11" s="2" t="n">
+        <v>112.998730099003</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>0.45058944405295</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>123.921828816043</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>0.45058944405295</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>201.478229776329</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0.700545785025913</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>18.9414485249961</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>0.675648581248717</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>-16.0542630817513</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>0.700545785025913</v>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>98.0726241598587</v>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>0.45058944405295</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>123.917489548646</v>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>0.45058944405295</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>45.8338521430273</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>0.700545785025913</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>-2.53922035909261</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>0.700545785025913</v>
+      </c>
+      <c r="T11" s="2" t="n">
+        <v>270.268424796213</v>
+      </c>
+      <c r="Y11" s="2" t="n">
+        <v>0.749644859282492</v>
+      </c>
+      <c r="Z11" s="2" t="n">
+        <v>134.765126340035</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C12" s="2" t="n">
+        <v>0.551214899264904</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>73.5860326902633</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>0.551214899264904</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>152.419027530903</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0.749644859282492</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>-0.123484941052084</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>0.551214899264904</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>73.5826129425848</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>0.551214899264904</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>63.2524374644692</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C13" s="2" t="n">
+        <v>0.650493343520364</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>30.3085884743077</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>0.650493343520364</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>56.0528799728351</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>0.650493343520364</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>30.3088206213848</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>0.650493343520364</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>67.7495174146844</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C14" s="2" t="n">
         <v>0.729293307111268</v>
       </c>
-      <c r="D11" s="0" t="n">
-        <v>16.6645455077503</v>
-      </c>
-      <c r="E11" s="2" t="n">
+      <c r="D14" s="2" t="n">
+        <v>16.5105545326853</v>
+      </c>
+      <c r="E14" s="2" t="n">
         <v>0.749644859282492</v>
       </c>
-      <c r="F11" s="0" t="n">
-        <v>-21.5201423238375</v>
-      </c>
-      <c r="G11" s="0" t="n">
-        <v>0.700545785025913</v>
-      </c>
-      <c r="H11" s="0" t="n">
-        <v>19.0754402376413</v>
-      </c>
-      <c r="I11" s="0" t="n">
+      <c r="F14" s="2" t="n">
+        <v>-21.1961215323112</v>
+      </c>
+      <c r="M14" s="2" t="n">
         <v>0.749644859282492</v>
       </c>
-      <c r="J11" s="0" t="n">
-        <v>-0.422608656101261</v>
-      </c>
-      <c r="K11" s="0" t="n">
-        <v>0.700545785025913</v>
-      </c>
-      <c r="L11" s="0" t="n">
-        <v>98.4987430862655</v>
-      </c>
-      <c r="M11" s="0" t="n">
+      <c r="N14" s="2" t="n">
+        <v>18.2234952062383</v>
+      </c>
+      <c r="O14" s="2" t="n">
         <v>0.749644859282492</v>
       </c>
-      <c r="N11" s="0" t="n">
-        <v>18.3416922138011</v>
-      </c>
-      <c r="O11" s="0" t="n">
-        <v>0.749644859282492</v>
-      </c>
-      <c r="P11" s="0" t="n">
-        <v>62.8946862975114</v>
-      </c>
-      <c r="Q11" s="0" t="n">
-        <v>0.700545785025913</v>
-      </c>
-      <c r="R11" s="0" t="n">
-        <v>-2.48018928734774</v>
-      </c>
-      <c r="S11" s="0" t="n">
-        <v>0.700545785025913</v>
-      </c>
-      <c r="T11" s="0" t="n">
-        <v>271.022200130503</v>
-      </c>
-      <c r="Y11" s="0" t="n">
-        <v>0.749644859282492</v>
-      </c>
-      <c r="Z11" s="0" t="n">
-        <v>142.603169549024</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C12" s="0" t="n">
-        <v>0.761787315617629</v>
-      </c>
-      <c r="D12" s="0" t="n">
-        <v>18.2349345149752</v>
-      </c>
-      <c r="E12" s="2" t="n">
+      <c r="P14" s="2" t="n">
+        <v>62.8142771757701</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C15" s="2" t="n">
         <v>0.801917215853616</v>
       </c>
-      <c r="F12" s="0" t="n">
-        <v>-35.5171084568784</v>
-      </c>
-      <c r="I12" s="0" t="n">
-        <v>0.801917215853616</v>
-      </c>
-      <c r="J12" s="0" t="n">
-        <v>23.7797963040628</v>
-      </c>
-      <c r="M12" s="0" t="n">
-        <v>0.801917215853616</v>
-      </c>
-      <c r="N12" s="0" t="n">
-        <v>32.0171603468683</v>
-      </c>
-      <c r="O12" s="0" t="n">
-        <v>0.801917215853616</v>
-      </c>
-      <c r="P12" s="0" t="n">
-        <v>51.7754063713867</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C13" s="0" t="n">
-        <v>0.801917215853616</v>
-      </c>
-      <c r="D13" s="0" t="n">
-        <v>23.8839581042439</v>
-      </c>
-      <c r="E13" s="2" t="n">
+      <c r="D15" s="2" t="n">
+        <v>23.872267714194</v>
+      </c>
+      <c r="E15" s="2" t="n">
         <v>0.849436782010227</v>
       </c>
-      <c r="F13" s="0" t="n">
-        <v>-27.4745755212531</v>
-      </c>
-      <c r="M13" s="0" t="n">
+      <c r="F15" s="2" t="n">
+        <v>-26.9052284996479</v>
+      </c>
+      <c r="M15" s="2" t="n">
         <v>0.849436782010227</v>
       </c>
-      <c r="N13" s="0" t="n">
-        <v>40.0445133788646</v>
-      </c>
-      <c r="O13" s="0" t="n">
+      <c r="N15" s="2" t="n">
+        <v>40.0556746315533</v>
+      </c>
+      <c r="O15" s="2" t="n">
         <v>0.849436782010227</v>
       </c>
-      <c r="P13" s="0" t="n">
-        <v>35.6056557712354</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C14" s="0" t="n">
-        <v>0.849436782010227</v>
-      </c>
-      <c r="D14" s="0" t="n">
-        <v>34.2563003232496</v>
-      </c>
-      <c r="E14" s="2" t="n">
+      <c r="P15" s="2" t="n">
+        <v>35.4548005268824</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C16" s="2" t="n">
         <v>0.900227517476009</v>
       </c>
-      <c r="F14" s="0" t="n">
-        <v>6.14495608435976</v>
-      </c>
-      <c r="M14" s="0" t="n">
-        <v>0.900227517476009</v>
-      </c>
-      <c r="N14" s="0" t="n">
-        <v>29.082538644202</v>
-      </c>
-      <c r="O14" s="0" t="n">
-        <v>0.900227517476009</v>
-      </c>
-      <c r="P14" s="0" t="n">
-        <v>18.5135026820109</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C15" s="0" t="n">
-        <v>0.900227517476009</v>
-      </c>
-      <c r="D15" s="0" t="n">
-        <v>46.1625681125523</v>
-      </c>
-      <c r="E15" s="2" t="n">
+      <c r="D16" s="2" t="n">
+        <v>46.4488802046767</v>
+      </c>
+      <c r="E16" s="2" t="n">
         <v>0.950390241271653</v>
       </c>
-      <c r="F15" s="0" t="n">
-        <v>64.4890620183401</v>
-      </c>
-      <c r="M15" s="0" t="n">
+      <c r="F16" s="2" t="n">
+        <v>64.6256541694259</v>
+      </c>
+      <c r="M16" s="2" t="n">
         <v>0.950390241271653</v>
       </c>
-      <c r="N15" s="0" t="n">
-        <v>10.10990383572</v>
-      </c>
-      <c r="O15" s="0" t="n">
+      <c r="N16" s="2" t="n">
+        <v>10.0766444952354</v>
+      </c>
+      <c r="O16" s="2" t="n">
         <v>0.950390241271653</v>
       </c>
-      <c r="P15" s="0" t="n">
-        <v>5.67755216973234</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C16" s="0" t="n">
-        <v>0.950390241271653</v>
-      </c>
-      <c r="D16" s="0" t="n">
-        <v>55.9281524527143</v>
-      </c>
-      <c r="E16" s="2" t="n">
+      <c r="P16" s="2" t="n">
+        <v>5.64892734720843</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="0" t="n">
-        <v>149.529064993417</v>
-      </c>
-      <c r="M16" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="N16" s="0" t="n">
-        <v>-0.0392911673076242</v>
-      </c>
-      <c r="O16" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="P16" s="0" t="n">
-        <v>-0.0392911673076242</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C17" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="0" t="n">
-        <v>63.5294553144536</v>
+      <c r="D17" s="2" t="n">
+        <v>63.9666008191205</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>